<commit_message>
Adjusted Deadlines and Added task 1
</commit_message>
<xml_diff>
--- a/CAB320 Work Split.xlsx
+++ b/CAB320 Work Split.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://connectqutedu-my.sharepoint.com/personal/n11285915_qut_edu_au/Documents/Documents/GitHub/CAB320-A2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="153" documentId="8_{95F0651F-E714-450A-BD31-BCF95EF3D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5EBE40D-A5C4-45AE-AA5B-3E8DA482E157}"/>
+  <xr:revisionPtr revIDLastSave="162" documentId="8_{95F0651F-E714-450A-BD31-BCF95EF3D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{167103F0-35EB-4EFB-A448-C6C50375C6F3}"/>
   <bookViews>
-    <workbookView xWindow="11505" yWindow="1560" windowWidth="22815" windowHeight="18165" xr2:uid="{15607E00-DA60-4B2F-9045-4CB7BAC65E04}"/>
+    <workbookView xWindow="10590" yWindow="0" windowWidth="27915" windowHeight="13395" xr2:uid="{15607E00-DA60-4B2F-9045-4CB7BAC65E04}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="125">
   <si>
     <t>Task No.</t>
   </si>
@@ -700,6 +700,12 @@
   </si>
   <si>
     <t>21-24 MAY</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>In Progress</t>
   </si>
 </sst>
 </file>
@@ -761,7 +767,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -798,6 +804,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -811,7 +829,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -822,9 +840,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -871,6 +886,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1215,8 +1245,8 @@
   <dimension ref="A1:J33"/>
   <sheetFormatPr defaultColWidth="36.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36.5703125" style="3"/>
     <col min="5" max="5" width="35.85546875" style="3" bestFit="1" customWidth="1"/>
@@ -1228,40 +1258,40 @@
     <col min="11" max="16384" width="36.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="8" customFormat="1">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:10" s="7" customFormat="1">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="45">
-      <c r="A2" s="10">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1288,12 +1318,12 @@
       <c r="I2" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J2" s="14" t="s">
-        <v>15</v>
+      <c r="J2" s="24" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30">
-      <c r="A3" s="10">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1320,30 +1350,30 @@
       <c r="I3" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J3" s="14" t="s">
-        <v>15</v>
+      <c r="J3" s="24" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="45">
-      <c r="A4" s="10">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H4" s="1">
@@ -1352,12 +1382,12 @@
       <c r="I4" s="2">
         <v>0.05</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="45">
-      <c r="A5" s="10">
+      <c r="A5" s="9">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1384,12 +1414,12 @@
       <c r="I5" s="2">
         <v>0.05</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>15</v>
+      <c r="J5" s="24" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="45">
-      <c r="A6" s="10">
+      <c r="A6" s="9">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1416,30 +1446,30 @@
       <c r="I6" s="2">
         <v>0.1</v>
       </c>
-      <c r="J6" s="14" t="s">
-        <v>15</v>
+      <c r="J6" s="24" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="45">
-      <c r="A7" s="10">
+      <c r="A7" s="9">
         <v>6</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H7" s="1">
@@ -1448,30 +1478,30 @@
       <c r="I7" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J7" s="14" t="s">
+      <c r="J7" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="45">
-      <c r="A8" s="10">
+      <c r="A8" s="9">
         <v>7</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="16" t="s">
+      <c r="G8" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H8" s="1">
@@ -1480,30 +1510,30 @@
       <c r="I8" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9" t="s">
+      <c r="A9" s="9"/>
+      <c r="B9" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="9">
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="8">
         <v>12</v>
       </c>
-      <c r="I9" s="20">
+      <c r="I9" s="19">
         <v>0.3</v>
       </c>
-      <c r="J9" s="10"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" spans="1:10" ht="42.75">
-      <c r="A10" s="10">
+      <c r="A10" s="9">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -1530,15 +1560,15 @@
       <c r="I10" s="2">
         <v>0.05</v>
       </c>
-      <c r="J10" s="14" t="s">
+      <c r="J10" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="45">
-      <c r="A11" s="10">
+      <c r="A11" s="9">
         <v>9</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>117</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1562,30 +1592,30 @@
       <c r="I11" s="2">
         <v>0.05</v>
       </c>
-      <c r="J11" s="14" t="s">
+      <c r="J11" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="45">
-      <c r="A12" s="10">
+      <c r="A12" s="9">
         <v>10</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="16" t="s">
+      <c r="G12" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H12" s="1">
@@ -1594,15 +1624,15 @@
       <c r="I12" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J12" s="14" t="s">
+      <c r="J12" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="30">
-      <c r="A13" s="10">
+      <c r="A13" s="9">
         <v>11</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>117</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -1626,30 +1656,30 @@
       <c r="I13" s="2">
         <v>0.05</v>
       </c>
-      <c r="J13" s="14" t="s">
+      <c r="J13" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="30">
-      <c r="A14" s="10">
+      <c r="A14" s="9">
         <v>12</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="16" t="s">
+      <c r="F14" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="16" t="s">
+      <c r="G14" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H14" s="1">
@@ -1658,15 +1688,15 @@
       <c r="I14" s="2">
         <v>0.05</v>
       </c>
-      <c r="J14" s="14" t="s">
+      <c r="J14" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="45">
-      <c r="A15" s="10">
+      <c r="A15" s="9">
         <v>13</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>117</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -1690,30 +1720,30 @@
       <c r="I15" s="2">
         <v>0.05</v>
       </c>
-      <c r="J15" s="14" t="s">
+      <c r="J15" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="45">
-      <c r="A16" s="10">
+      <c r="A16" s="9">
         <v>14</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="E16" s="16" t="s">
+      <c r="E16" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="F16" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G16" s="16" t="s">
+      <c r="G16" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H16" s="1">
@@ -1722,30 +1752,30 @@
       <c r="I16" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J16" s="14" t="s">
+      <c r="J16" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="10"/>
-      <c r="B17" s="9" t="s">
+      <c r="A17" s="9"/>
+      <c r="B17" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="9">
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="8">
         <v>12</v>
       </c>
-      <c r="I17" s="20">
+      <c r="I17" s="19">
         <v>0.3</v>
       </c>
-      <c r="J17" s="10"/>
+      <c r="J17" s="9"/>
     </row>
     <row r="18" spans="1:10" ht="30">
-      <c r="A18" s="10">
+      <c r="A18" s="9">
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -1772,12 +1802,12 @@
       <c r="I18" s="2">
         <v>0.05</v>
       </c>
-      <c r="J18" s="14" t="s">
+      <c r="J18" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="30">
-      <c r="A19" s="10">
+      <c r="A19" s="9">
         <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1804,30 +1834,30 @@
       <c r="I19" s="2">
         <v>0.05</v>
       </c>
-      <c r="J19" s="14" t="s">
+      <c r="J19" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="45">
-      <c r="A20" s="10">
+      <c r="A20" s="9">
         <v>17</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="E20" s="16" t="s">
+      <c r="E20" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="F20" s="16" t="s">
+      <c r="F20" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="G20" s="16" t="s">
+      <c r="G20" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H20" s="1">
@@ -1836,12 +1866,12 @@
       <c r="I20" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J20" s="14" t="s">
+      <c r="J20" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="30">
-      <c r="A21" s="10">
+      <c r="A21" s="9">
         <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1868,30 +1898,30 @@
       <c r="I21" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J21" s="14" t="s">
+      <c r="J21" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="45">
-      <c r="A22" s="10">
+      <c r="A22" s="9">
         <v>19</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="E22" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="F22" s="16" t="s">
+      <c r="F22" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H22" s="1">
@@ -1900,12 +1930,12 @@
       <c r="I22" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J22" s="14" t="s">
+      <c r="J22" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="45">
-      <c r="A23" s="10">
+      <c r="A23" s="9">
         <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -1932,30 +1962,30 @@
       <c r="I23" s="2">
         <v>0.1</v>
       </c>
-      <c r="J23" s="14" t="s">
+      <c r="J23" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="45">
-      <c r="A24" s="10">
+      <c r="A24" s="9">
         <v>21</v>
       </c>
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="16" t="s">
+      <c r="D24" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="E24" s="16" t="s">
+      <c r="E24" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="F24" s="16" t="s">
+      <c r="F24" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="G24" s="16" t="s">
+      <c r="G24" s="15" t="s">
         <v>121</v>
       </c>
       <c r="H24" s="1">
@@ -1964,12 +1994,12 @@
       <c r="I24" s="2">
         <v>0.05</v>
       </c>
-      <c r="J24" s="14" t="s">
+      <c r="J24" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="45">
-      <c r="A25" s="10">
+      <c r="A25" s="9">
         <v>22</v>
       </c>
       <c r="B25" s="1" t="s">
@@ -1996,102 +2026,106 @@
       <c r="I25" s="2">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="J25" s="14" t="s">
+      <c r="J25" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:10">
-      <c r="A26" s="10"/>
-      <c r="B26" s="9" t="s">
+      <c r="A26" s="9"/>
+      <c r="B26" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="9">
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="8">
         <v>16</v>
       </c>
-      <c r="I26" s="20">
+      <c r="I26" s="19">
         <v>0.4</v>
       </c>
-      <c r="J26" s="10"/>
+      <c r="J26" s="9"/>
     </row>
     <row r="28" spans="1:10">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="10" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="29" spans="1:10">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="9" t="s">
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H29" s="12"/>
-      <c r="I29" s="12"/>
-      <c r="J29" s="9" t="s">
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="75">
-      <c r="A30" s="10">
+      <c r="A30" s="9">
         <v>23</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="G30" s="17">
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="23">
         <v>46162</v>
       </c>
-      <c r="J30" s="14" t="s">
+      <c r="H30" s="22"/>
+      <c r="I30" s="22"/>
+      <c r="J30" s="20" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="30">
+      <c r="A31" s="9">
+        <v>24</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="F31" s="18"/>
+      <c r="G31" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="H31" s="18"/>
+      <c r="I31" s="18"/>
+      <c r="J31" s="17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="30">
-      <c r="A31" s="10">
-        <v>24</v>
-      </c>
-      <c r="B31" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="C31" s="18" t="s">
-        <v>108</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>109</v>
-      </c>
-      <c r="F31" s="19"/>
-      <c r="G31" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="H31" s="19"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="18" t="s">
-        <v>15</v>
-      </c>
-    </row>
     <row r="32" spans="1:10" ht="45">
-      <c r="A32" s="10">
+      <c r="A32" s="9">
         <v>25</v>
       </c>
       <c r="B32" s="1" t="s">
@@ -2103,15 +2137,15 @@
       <c r="D32" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="G32" s="17">
+      <c r="G32" s="16">
         <v>46168</v>
       </c>
-      <c r="J32" s="14" t="s">
+      <c r="J32" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="30">
-      <c r="A33" s="10">
+      <c r="A33" s="9">
         <v>26</v>
       </c>
       <c r="B33" s="1" t="s">
@@ -2123,10 +2157,10 @@
       <c r="D33" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="G33" s="17">
+      <c r="G33" s="16">
         <v>46171</v>
       </c>
-      <c r="J33" s="14" t="s">
+      <c r="J33" s="13" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated Sub Task Statuses
</commit_message>
<xml_diff>
--- a/CAB320 Work Split.xlsx
+++ b/CAB320 Work Split.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://connectqutedu-my.sharepoint.com/personal/n11285915_qut_edu_au/Documents/Documents/GitHub/CAB320-A2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="162" documentId="8_{95F0651F-E714-450A-BD31-BCF95EF3D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{167103F0-35EB-4EFB-A448-C6C50375C6F3}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="8_{95F0651F-E714-450A-BD31-BCF95EF3D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{855E250F-1035-4CAF-A9A5-612D2DEF1884}"/>
   <bookViews>
     <workbookView xWindow="10590" yWindow="0" windowWidth="27915" windowHeight="13395" xr2:uid="{15607E00-DA60-4B2F-9045-4CB7BAC65E04}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="126">
   <si>
     <t>Task No.</t>
   </si>
@@ -706,6 +706,9 @@
   </si>
   <si>
     <t>In Progress</t>
+  </si>
+  <si>
+    <t>Complete</t>
   </si>
 </sst>
 </file>
@@ -829,7 +832,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -901,6 +904,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1246,7 +1255,7 @@
   <sheetFormatPr defaultColWidth="36.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36.5703125" style="3"/>
     <col min="5" max="5" width="35.85546875" style="3" bestFit="1" customWidth="1"/>
@@ -1258,7 +1267,7 @@
     <col min="11" max="16384" width="36.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="7" customFormat="1">
+    <row r="1" spans="1:10" s="7" customFormat="1" ht="30">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1294,96 +1303,96 @@
       <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="20">
         <v>1</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="25">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J2" s="24" t="s">
-        <v>124</v>
+      <c r="J2" s="20" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30">
       <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="20">
         <v>1</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="25">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J3" s="24" t="s">
-        <v>124</v>
+      <c r="J3" s="20" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="45">
       <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="20">
         <v>2</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="25">
         <v>0.05</v>
       </c>
-      <c r="J4" s="13" t="s">
-        <v>15</v>
+      <c r="J4" s="20" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="45">

</xml_diff>

<commit_message>
Updated Completed Section 1
</commit_message>
<xml_diff>
--- a/CAB320 Work Split.xlsx
+++ b/CAB320 Work Split.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://connectqutedu-my.sharepoint.com/personal/n11285915_qut_edu_au/Documents/Documents/GitHub/CAB320-A2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="8_{95F0651F-E714-450A-BD31-BCF95EF3D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{855E250F-1035-4CAF-A9A5-612D2DEF1884}"/>
+  <xr:revisionPtr revIDLastSave="180" documentId="8_{95F0651F-E714-450A-BD31-BCF95EF3D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49B80925-1068-4227-9776-89F5AAE007FF}"/>
   <bookViews>
-    <workbookView xWindow="10590" yWindow="0" windowWidth="27915" windowHeight="13395" xr2:uid="{15607E00-DA60-4B2F-9045-4CB7BAC65E04}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{15607E00-DA60-4B2F-9045-4CB7BAC65E04}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="125">
   <si>
     <t>Task No.</t>
   </si>
@@ -665,12 +665,31 @@
     <t>Joshua Oates</t>
   </si>
   <si>
+    <t>25-27 MAY</t>
+  </si>
+  <si>
+    <t>18-21 MAY</t>
+  </si>
+  <si>
+    <t>27-29 MAY</t>
+  </si>
+  <si>
+    <t>21-24 MAY</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Explain how </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <strike/>
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
@@ -680,6 +699,7 @@
     <r>
       <rPr>
         <b/>
+        <strike/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
@@ -688,34 +708,13 @@
       </rPr>
       <t xml:space="preserve"> works</t>
     </r>
-  </si>
-  <si>
-    <t>25-27 MAY</t>
-  </si>
-  <si>
-    <t>18-21 MAY</t>
-  </si>
-  <si>
-    <t>27-29 MAY</t>
-  </si>
-  <si>
-    <t>21-24 MAY</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>Complete</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -756,18 +755,28 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Unicode MS"/>
-    </font>
-    <font>
       <strike/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="9">
@@ -815,7 +824,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -832,7 +841,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -882,10 +891,10 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -903,13 +912,19 @@
     <xf numFmtId="16" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="10" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1267,7 +1282,7 @@
     <col min="11" max="16384" width="36.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="7" customFormat="1" ht="30">
+    <row r="1" spans="1:10" s="7" customFormat="1">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1319,16 +1334,16 @@
         <v>13</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H2" s="20">
         <v>1</v>
       </c>
-      <c r="I2" s="25">
+      <c r="I2" s="24">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30">
@@ -1351,143 +1366,143 @@
         <v>19</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H3" s="20">
         <v>1</v>
       </c>
-      <c r="I3" s="25">
+      <c r="I3" s="24">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="J3" s="20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="45">
       <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="E4" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="26" t="s">
-        <v>121</v>
+      <c r="G4" s="25" t="s">
+        <v>120</v>
       </c>
       <c r="H4" s="20">
         <v>2</v>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="24">
         <v>0.05</v>
       </c>
       <c r="J4" s="20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="45">
       <c r="A5" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="H5" s="1">
+      <c r="G5" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="H5" s="20">
         <v>2</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="24">
         <v>0.05</v>
       </c>
-      <c r="J5" s="24" t="s">
-        <v>124</v>
+      <c r="J5" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="45">
       <c r="A6" s="9">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="H6" s="1">
+      <c r="G6" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="H6" s="20">
         <v>4</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="24">
         <v>0.1</v>
       </c>
-      <c r="J6" s="24" t="s">
-        <v>124</v>
+      <c r="J6" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="45">
       <c r="A7" s="9">
         <v>6</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="E7" s="15" t="s">
+      <c r="D7" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="E7" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="H7" s="1">
+      <c r="G7" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="H7" s="27">
         <v>1</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="28">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="J7" s="27" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1511,7 +1526,7 @@
         <v>38</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H8" s="1">
         <v>1</v>
@@ -1545,32 +1560,32 @@
       <c r="A10" s="9">
         <v>8</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="B10" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="H10" s="1">
+      <c r="G10" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="H10" s="20">
         <v>2</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="24">
         <v>0.05</v>
       </c>
-      <c r="J10" s="13" t="s">
-        <v>15</v>
+      <c r="J10" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="45">
@@ -1593,7 +1608,7 @@
         <v>46</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H11" s="1">
         <v>2</v>
@@ -1625,7 +1640,7 @@
         <v>50</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H12" s="1">
         <v>1</v>
@@ -1657,7 +1672,7 @@
         <v>54</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H13" s="1">
         <v>2</v>
@@ -1689,7 +1704,7 @@
         <v>58</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H14" s="1">
         <v>2</v>
@@ -1721,7 +1736,7 @@
         <v>62</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H15" s="1">
         <v>2</v>
@@ -1753,7 +1768,7 @@
         <v>66</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H16" s="1">
         <v>1</v>
@@ -1803,7 +1818,7 @@
         <v>71</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H18" s="1">
         <v>2</v>
@@ -1835,7 +1850,7 @@
         <v>75</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H19" s="1">
         <v>2</v>
@@ -1867,7 +1882,7 @@
         <v>79</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H20" s="1">
         <v>1</v>
@@ -1899,7 +1914,7 @@
         <v>83</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H21" s="1">
         <v>1</v>
@@ -1931,7 +1946,7 @@
         <v>87</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H22" s="1">
         <v>1</v>
@@ -1963,7 +1978,7 @@
         <v>91</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H23" s="1">
         <v>4</v>
@@ -1995,7 +2010,7 @@
         <v>95</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H24" s="1">
         <v>2</v>
@@ -2027,7 +2042,7 @@
         <v>99</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H25" s="1">
         <v>3</v>
@@ -2107,7 +2122,7 @@
       <c r="H30" s="22"/>
       <c r="I30" s="22"/>
       <c r="J30" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="30">

</xml_diff>

<commit_message>
Fixed Main File Issue, Updated worksheet
Fixed task 7-9 visibility following a push error with oates branch
</commit_message>
<xml_diff>
--- a/CAB320 Work Split.xlsx
+++ b/CAB320 Work Split.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://connectqutedu-my.sharepoint.com/personal/n11285915_qut_edu_au/Documents/Documents/GitHub/CAB320-A2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="180" documentId="8_{95F0651F-E714-450A-BD31-BCF95EF3D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49B80925-1068-4227-9776-89F5AAE007FF}"/>
+  <xr:revisionPtr revIDLastSave="200" documentId="8_{95F0651F-E714-450A-BD31-BCF95EF3D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5173942-F1AA-4178-BDE0-C5215A4AFDF8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{15607E00-DA60-4B2F-9045-4CB7BAC65E04}"/>
+    <workbookView xWindow="-28920" yWindow="1965" windowWidth="29040" windowHeight="15720" xr2:uid="{15607E00-DA60-4B2F-9045-4CB7BAC65E04}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -841,7 +841,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -926,6 +926,9 @@
     </xf>
     <xf numFmtId="10" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1592,63 +1595,63 @@
       <c r="A11" s="9">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="20">
         <v>2</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="24">
         <v>0.05</v>
       </c>
-      <c r="J11" s="13" t="s">
-        <v>15</v>
+      <c r="J11" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="45">
       <c r="A12" s="9">
         <v>10</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="G12" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="26">
         <v>1</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="26">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J12" s="13" t="s">
+      <c r="J12" s="26" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1656,64 +1659,64 @@
       <c r="A13" s="9">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="20">
         <v>2</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="24">
         <v>0.05</v>
       </c>
-      <c r="J13" s="13" t="s">
-        <v>15</v>
+      <c r="J13" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="30">
       <c r="A14" s="9">
         <v>12</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="G14" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="20">
         <v>2</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="24">
         <v>0.05</v>
       </c>
-      <c r="J14" s="13" t="s">
-        <v>15</v>
+      <c r="J14" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="45">
@@ -1744,8 +1747,8 @@
       <c r="I15" s="2">
         <v>0.05</v>
       </c>
-      <c r="J15" s="13" t="s">
-        <v>15</v>
+      <c r="J15" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="45">

</xml_diff>